<commit_message>
updated with Medium Fixed
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{503F0908-0BD5-49ED-944D-01DDD0EE280F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC072377-3E44-4860-965A-C19C780C9721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -247,7 +247,7 @@
     <t>CI/CD</t>
   </si>
   <si>
-    <t>C:\Users\srina1k\Downloads\Automation TestData\Data_S1_AT.csv</t>
+    <t>C:\Users\srina1k\OneDrive - EDF\Data_S1_JAN_RT.csv</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
updated with Medium Fixed -P1
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC072377-3E44-4860-965A-C19C780C9721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B73FD1-4A37-46E9-9719-A00EA65EE7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,9 +94,6 @@
     <t>9447764380</t>
   </si>
   <si>
-    <t>D:\\Users\\sunag1a\\RTInputFiles\\Data_S7_RT.csv</t>
-  </si>
-  <si>
     <t>Customer_Name</t>
   </si>
   <si>
@@ -248,6 +245,9 @@
   </si>
   <si>
     <t>C:\Users\srina1k\OneDrive - EDF\Data_S1_JAN_RT.csv</t>
+  </si>
+  <si>
+    <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S7_RT.csv</t>
   </si>
 </sst>
 </file>
@@ -898,7 +898,7 @@
         <v>12</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -924,13 +924,13 @@
         <v>3482055476</v>
       </c>
       <c r="H3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -938,14 +938,14 @@
         <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -953,106 +953,106 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="H5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D6" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="H6" s="2">
-        <v>5463584629</v>
+        <v>7825449437</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="J7" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="I9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="J9" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="I10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H11" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J11" s="7"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G12" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H12" s="2">
         <v>7641311796</v>
@@ -1060,7 +1060,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G13" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H13" s="2">
         <v>9065870431</v>
@@ -1068,7 +1068,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G14" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H14" s="2">
         <v>4376617890</v>
@@ -1076,53 +1076,53 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G16" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="17" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G17" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G18" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G19" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G20" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G21" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G22" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H22" s="2"/>
     </row>
@@ -1173,45 +1173,45 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>61</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B2" s="11"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B3" s="11"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="11"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B6" s="11"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B7" s="11"/>
     </row>

</xml_diff>

<commit_message>
updated with Medium Fixed Test Run
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B73FD1-4A37-46E9-9719-A00EA65EE7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3389AC25-BB48-4BBA-BC16-7A3578340D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -244,16 +244,23 @@
     <t>CI/CD</t>
   </si>
   <si>
-    <t>C:\Users\srina1k\OneDrive - EDF\Data_S1_JAN_RT.csv</t>
-  </si>
-  <si>
-    <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S7_RT.csv</t>
+    <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S1_JAN_RT.csv</t>
+  </si>
+  <si>
+    <t>C:\\Users\\srina1k\\Downloads\\Data_S7_RT.csv</t>
+  </si>
+  <si>
+    <t>4450634772</t>
+  </si>
+  <si>
+    <t>0635298882</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -831,16 +838,16 @@
   <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.140625" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="2" max="2" customWidth="true" width="15.0"/>
+    <col min="3" max="3" customWidth="true" width="12.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="14.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="52.140625"/>
+    <col min="6" max="6" customWidth="true" width="17.140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="20.140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="51.28515625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="47.5703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -923,7 +930,7 @@
       <c r="G3" s="2">
         <v>3482055476</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" t="s" s="0">
         <v>69</v>
       </c>
       <c r="I3" s="6" t="s">
@@ -968,7 +975,7 @@
         <v>27</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>23</v>
@@ -1143,7 +1150,7 @@
   <dimension ref="C1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
@@ -1167,8 +1174,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.140625" customWidth="1"/>
-    <col min="2" max="2" width="56.28515625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="28.140625"/>
+    <col min="2" max="2" customWidth="true" width="56.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated with Flex-Basket - p1
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47B5A49-1BF9-403B-BE64-440BB7A2AD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6EDFB6-8064-4C50-B52A-6C0BE20443CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="85">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -160,15 +160,9 @@
     <t>Customer Upload file</t>
   </si>
   <si>
-    <t>D:\\Users\\sunag1a\\RTInputFiles\\S-12-CM-CUUB2.csv</t>
-  </si>
-  <si>
     <t>Bulk Opp Uplaod</t>
   </si>
   <si>
-    <t>D:\\Users\\sunag1a\\RTInputFiles\\S-12-CMBLRNOP.csv</t>
-  </si>
-  <si>
     <t>Opp ID-1</t>
   </si>
   <si>
@@ -214,82 +208,91 @@
     <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S1_JAN_RT.csv</t>
   </si>
   <si>
-    <t>C:\\Users\\srina1k\\Downloads\\Data_S7_RT.csv</t>
-  </si>
-  <si>
-    <t>0108766516</t>
-  </si>
-  <si>
     <t>1234617877</t>
   </si>
   <si>
     <t>7108788894</t>
   </si>
   <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\S19_2.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\S19_3.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\S19_4.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_1_DEC_MCT 1.txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_2_DEC_MCT 1.txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_3_DEC_MCT 1.txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_4_DEC_MCT 1.txt</t>
-  </si>
-  <si>
-    <t>7903110159</t>
-  </si>
-  <si>
     <t>1560000000</t>
   </si>
   <si>
-    <t>3182723121</t>
-  </si>
-  <si>
-    <t>1577163529</t>
-  </si>
-  <si>
-    <t>4339230149</t>
-  </si>
-  <si>
-    <t>0139180146</t>
-  </si>
-  <si>
-    <t>2652616891</t>
-  </si>
-  <si>
-    <t>9563151772</t>
-  </si>
-  <si>
-    <t>0598076921</t>
-  </si>
-  <si>
-    <t>0461612620</t>
-  </si>
-  <si>
-    <t>8559102288</t>
-  </si>
-  <si>
-    <t>3525610539</t>
-  </si>
-  <si>
-    <t>7342369718</t>
-  </si>
-  <si>
-    <t>1580018346</t>
-  </si>
-  <si>
-    <t>5076940279</t>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation2.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation3.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MediumFixed-p1\\Data_S7_RT.csv</t>
+  </si>
+  <si>
+    <t>Framework Id</t>
+  </si>
+  <si>
+    <t>1118518080</t>
+  </si>
+  <si>
+    <t>7007727568</t>
+  </si>
+  <si>
+    <t>0245182125</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\FlexBasket - P1\\CUUB2-BATCH-25-03-2026.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\FlexBasket - P1\\CMBLRNOP_S12_FLEX_ADDSITE_18JUNE-2025 RT.csv</t>
+  </si>
+  <si>
+    <t>4830919677</t>
+  </si>
+  <si>
+    <t>2985832464</t>
+  </si>
+  <si>
+    <t>0070458779</t>
+  </si>
+  <si>
+    <t>6617429933</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_1_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\AutomationDocuments\MCTOpportunity\OPP_2_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_3_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_4_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>1798345198</t>
+  </si>
+  <si>
+    <t>3263251768</t>
+  </si>
+  <si>
+    <t>1440805649</t>
+  </si>
+  <si>
+    <t>6330372490</t>
+  </si>
+  <si>
+    <t>5487542683</t>
+  </si>
+  <si>
+    <t>3965168945</t>
+  </si>
+  <si>
+    <t>0004921201</t>
+  </si>
+  <si>
+    <t>9852945720</t>
   </si>
 </sst>
 </file>
@@ -297,7 +300,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -349,6 +352,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -385,7 +396,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -401,6 +412,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -871,7 +883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.7109375"/>
@@ -896,21 +908,21 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9" t="s">
+      <c r="E1" s="10"/>
+      <c r="F1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9"/>
+      <c r="G1" s="10"/>
       <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="9"/>
+      <c r="J1" s="10"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -926,7 +938,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2">
         <v>3151000000</v>
@@ -941,7 +953,7 @@
         <v>11</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -958,7 +970,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" s="2">
         <v>2280000000</v>
@@ -967,7 +979,7 @@
         <v>3482055476</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>16</v>
@@ -988,11 +1000,13 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
@@ -1008,10 +1022,10 @@
         <v>23</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>20</v>
@@ -1025,10 +1039,10 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H6" s="2">
-        <v>7825449437</v>
+        <v>9464875473</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -1036,7 +1050,7 @@
         <v>26</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>27</v>
@@ -1047,7 +1061,7 @@
         <v>28</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>7</v>
@@ -1061,13 +1075,13 @@
         <v>30</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>31</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1075,7 +1089,7 @@
         <v>32</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>33</v>
@@ -1092,7 +1106,7 @@
         <v>20</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1124,52 +1138,65 @@
         <v>39</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G16" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G17" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="18" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G18" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H18" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="19" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G19" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H19" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="20" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G20" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H20" s="2"/>
+        <v>63</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="21" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G21" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G22" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="H22" s="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G23" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="H23" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1192,11 +1219,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1218,47 +1245,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>50</v>
+        <v>47</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="11"/>
+        <v>49</v>
+      </c>
+      <c r="B2" s="12"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" s="11"/>
+        <v>50</v>
+      </c>
+      <c r="B3" s="12"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="11"/>
+        <v>51</v>
+      </c>
+      <c r="B4" s="12"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="11"/>
+        <v>52</v>
+      </c>
+      <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="11"/>
+        <v>53</v>
+      </c>
+      <c r="B6" s="12"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="11"/>
+        <v>54</v>
+      </c>
+      <c r="B7" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
updated with pdv & Overdue
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6EDFB6-8064-4C50-B52A-6C0BE20443CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10811F00-2D88-429F-97BC-0A82B056DFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -214,85 +214,103 @@
     <t>7108788894</t>
   </si>
   <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation2.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation3.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MediumFixed-p1\\Data_S7_RT.csv</t>
+  </si>
+  <si>
+    <t>Framework Id</t>
+  </si>
+  <si>
+    <t>7007727568</t>
+  </si>
+  <si>
+    <t>0245182125</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_1_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\AutomationDocuments\MCTOpportunity\OPP_2_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_3_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_4_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CM-CUUB2_FLEX_BASKET_BV_30MAR2025 RT-BATCH 1.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CMBLRNOP_S12_FLEX_ADDSITE_30March-2025 RT.csv</t>
+  </si>
+  <si>
+    <t>3705918716</t>
+  </si>
+  <si>
+    <t>8281545666</t>
+  </si>
+  <si>
+    <t>6272226556</t>
+  </si>
+  <si>
+    <t>9930714757</t>
+  </si>
+  <si>
+    <t>5313210615</t>
+  </si>
+  <si>
     <t>1560000000</t>
   </si>
   <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation2.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation3.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MediumFixed-p1\\Data_S7_RT.csv</t>
-  </si>
-  <si>
-    <t>Framework Id</t>
-  </si>
-  <si>
-    <t>1118518080</t>
-  </si>
-  <si>
-    <t>7007727568</t>
-  </si>
-  <si>
-    <t>0245182125</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\FlexBasket - P1\\CUUB2-BATCH-25-03-2026.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\FlexBasket - P1\\CMBLRNOP_S12_FLEX_ADDSITE_18JUNE-2025 RT.csv</t>
-  </si>
-  <si>
-    <t>4830919677</t>
-  </si>
-  <si>
-    <t>2985832464</t>
-  </si>
-  <si>
-    <t>0070458779</t>
-  </si>
-  <si>
-    <t>6617429933</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_1_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\AutomationDocuments\MCTOpportunity\OPP_2_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_3_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_4_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>1798345198</t>
-  </si>
-  <si>
-    <t>3263251768</t>
-  </si>
-  <si>
-    <t>1440805649</t>
-  </si>
-  <si>
-    <t>6330372490</t>
-  </si>
-  <si>
-    <t>5487542683</t>
-  </si>
-  <si>
-    <t>3965168945</t>
-  </si>
-  <si>
-    <t>0004921201</t>
-  </si>
-  <si>
-    <t>9852945720</t>
+    <t>6157738581</t>
+  </si>
+  <si>
+    <t>5477397575</t>
+  </si>
+  <si>
+    <t>6787561103</t>
+  </si>
+  <si>
+    <t>3924439311</t>
+  </si>
+  <si>
+    <t>0596362331</t>
+  </si>
+  <si>
+    <t>5122638063</t>
+  </si>
+  <si>
+    <t>0876646862</t>
+  </si>
+  <si>
+    <t>6579077315</t>
+  </si>
+  <si>
+    <t>8525362589</t>
+  </si>
+  <si>
+    <t>4565185268</t>
+  </si>
+  <si>
+    <t>6770510767</t>
+  </si>
+  <si>
+    <t>7730327480</t>
+  </si>
+  <si>
+    <t>8250985049</t>
+  </si>
+  <si>
+    <t>2633799055</t>
   </si>
 </sst>
 </file>
@@ -938,7 +956,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="F2" s="2">
         <v>3151000000</v>
@@ -970,7 +988,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F3" s="2">
         <v>2280000000</v>
@@ -979,7 +997,7 @@
         <v>3482055476</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>16</v>
@@ -1000,12 +1018,12 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1022,10 +1040,10 @@
         <v>23</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>20</v>
@@ -1039,7 +1057,7 @@
         <v>25</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H6" s="2">
         <v>9464875473</v>
@@ -1050,7 +1068,7 @@
         <v>26</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>27</v>
@@ -1061,7 +1079,7 @@
         <v>28</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>7</v>
@@ -1075,13 +1093,13 @@
         <v>30</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>31</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1089,7 +1107,7 @@
         <v>32</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>33</v>
@@ -1106,7 +1124,7 @@
         <v>20</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>57</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1138,7 +1156,7 @@
         <v>39</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1146,7 +1164,7 @@
         <v>40</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="7:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1172,7 @@
         <v>41</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="7:8" x14ac:dyDescent="0.25">
@@ -1162,7 +1180,7 @@
         <v>42</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="7:8" x14ac:dyDescent="0.25">
@@ -1170,15 +1188,15 @@
         <v>43</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G20" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="7:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update with some ignored files
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="93">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -311,6 +311,12 @@
   </si>
   <si>
     <t>2633799055</t>
+  </si>
+  <si>
+    <t>1542461040</t>
+  </si>
+  <si>
+    <t>5356202583</t>
   </si>
 </sst>
 </file>
@@ -1011,7 +1017,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>18</v>
+        <v>92</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="5" t="s">

</xml_diff>

<commit_message>
updated with live billing P1
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10811F00-2D88-429F-97BC-0A82B056DFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25EBB01-39ED-41F3-A92D-9642B765FCFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="92">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -94,9 +94,6 @@
     <t>CARPENTER INVESTMENTS (VINE STREET) LTD</t>
   </si>
   <si>
-    <t>9685173917</t>
-  </si>
-  <si>
     <t>CSV_File_1</t>
   </si>
   <si>
@@ -208,12 +205,6 @@
     <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S1_JAN_RT.csv</t>
   </si>
   <si>
-    <t>1234617877</t>
-  </si>
-  <si>
-    <t>7108788894</t>
-  </si>
-  <si>
     <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
   </si>
   <si>
@@ -229,9 +220,6 @@
     <t>Framework Id</t>
   </si>
   <si>
-    <t>7007727568</t>
-  </si>
-  <si>
     <t>0245182125</t>
   </si>
   <si>
@@ -253,45 +241,9 @@
     <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CMBLRNOP_S12_FLEX_ADDSITE_30March-2025 RT.csv</t>
   </si>
   <si>
-    <t>3705918716</t>
-  </si>
-  <si>
-    <t>8281545666</t>
-  </si>
-  <si>
-    <t>6272226556</t>
-  </si>
-  <si>
-    <t>9930714757</t>
-  </si>
-  <si>
-    <t>5313210615</t>
-  </si>
-  <si>
     <t>1560000000</t>
   </si>
   <si>
-    <t>6157738581</t>
-  </si>
-  <si>
-    <t>5477397575</t>
-  </si>
-  <si>
-    <t>6787561103</t>
-  </si>
-  <si>
-    <t>3924439311</t>
-  </si>
-  <si>
-    <t>0596362331</t>
-  </si>
-  <si>
-    <t>5122638063</t>
-  </si>
-  <si>
-    <t>0876646862</t>
-  </si>
-  <si>
     <t>6579077315</t>
   </si>
   <si>
@@ -313,10 +265,55 @@
     <t>2633799055</t>
   </si>
   <si>
-    <t>1542461040</t>
-  </si>
-  <si>
-    <t>5356202583</t>
+    <t>5149622225</t>
+  </si>
+  <si>
+    <t>7777857402</t>
+  </si>
+  <si>
+    <t>Live Billing P1</t>
+  </si>
+  <si>
+    <t>Live Billing</t>
+  </si>
+  <si>
+    <t>Person_ID-1</t>
+  </si>
+  <si>
+    <t>Child Person ID</t>
+  </si>
+  <si>
+    <t>OPP_ID</t>
+  </si>
+  <si>
+    <t>NHH MPAN</t>
+  </si>
+  <si>
+    <t>HH MPAN</t>
+  </si>
+  <si>
+    <t>1502000000</t>
+  </si>
+  <si>
+    <t>5433000000</t>
+  </si>
+  <si>
+    <t>9574256063</t>
+  </si>
+  <si>
+    <t>6923383318</t>
+  </si>
+  <si>
+    <t>9759372210</t>
+  </si>
+  <si>
+    <t>0731479811</t>
+  </si>
+  <si>
+    <t>2696403742</t>
+  </si>
+  <si>
+    <t>2088160177</t>
   </si>
 </sst>
 </file>
@@ -324,7 +321,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -384,6 +381,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF856EC6"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -420,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -433,10 +437,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -446,12 +452,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF856EC6"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -907,7 +921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.7109375"/>
@@ -920,9 +934,12 @@
     <col min="8" max="8" bestFit="true" customWidth="true" width="51.28515625"/>
     <col min="9" max="9" bestFit="true" customWidth="true" width="16.0"/>
     <col min="10" max="10" bestFit="true" customWidth="true" width="47.5703125"/>
+    <col min="12" max="12" customWidth="true" width="5.85546875"/>
+    <col min="13" max="14" customWidth="true" hidden="true" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" width="24.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -932,23 +949,26 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10" t="s">
+      <c r="E1" s="12"/>
+      <c r="F1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="10"/>
+      <c r="G1" s="12"/>
       <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="10"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J1" s="12"/>
+      <c r="O1" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
@@ -961,8 +981,8 @@
       <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>76</v>
+      <c r="E2" s="15" t="s">
+        <v>67</v>
       </c>
       <c r="F2" s="2">
         <v>3151000000</v>
@@ -977,10 +997,10 @@
         <v>11</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
@@ -994,7 +1014,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="F3" s="2">
         <v>2280000000</v>
@@ -1003,7 +1023,7 @@
         <v>3482055476</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>16</v>
@@ -1012,213 +1032,247 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D6" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="2">
+        <v>7007727568</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="2">
-        <v>9464875473</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="J7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D8" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D8" s="5" t="s">
-        <v>28</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D9" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D10" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J9" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I10" s="5" t="s">
+      <c r="J10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="J10" s="6" t="s">
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H11" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G12" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G12" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="H12" s="2">
         <v>7641311796</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D13" s="1"/>
+      <c r="E13" s="10" t="s">
+        <v>78</v>
+      </c>
       <c r="G13" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H13" s="2">
         <v>9065870431</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D14" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>84</v>
+      </c>
       <c r="G14" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H14" s="2">
         <v>4376617890</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D15" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="G15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D16" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G16" s="5" t="s">
+      <c r="H16" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D17" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E17" s="11">
+        <v>1591062611809</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G17" s="5" t="s">
+      <c r="H17" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D18" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="11">
+        <v>1600000042214</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G19" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G20" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G21" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G20" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="21" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G21" s="5" t="s">
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G22" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G22" s="5" t="s">
+    </row>
+    <row r="23" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="G23" s="8" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G23" s="9" t="s">
-        <v>46</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -1243,11 +1297,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1269,47 +1323,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>47</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" s="12"/>
+        <v>48</v>
+      </c>
+      <c r="B2" s="14"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="12"/>
+        <v>49</v>
+      </c>
+      <c r="B3" s="14"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="12"/>
+        <v>50</v>
+      </c>
+      <c r="B4" s="14"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="12"/>
+        <v>51</v>
+      </c>
+      <c r="B5" s="14"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="12"/>
+        <v>52</v>
+      </c>
+      <c r="B6" s="14"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="12"/>
+        <v>53</v>
+      </c>
+      <c r="B7" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
updated with COT P2 & Medium Fixed P2
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25EBB01-39ED-41F3-A92D-9642B765FCFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1890684E-1950-4984-9E00-5D3817C51ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="95">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -70,400 +70,259 @@
     <t>5021406696</t>
   </si>
   <si>
+    <t>UploadingFile</t>
+  </si>
+  <si>
+    <t>Premise_ID</t>
+  </si>
+  <si>
+    <t>7637797801</t>
+  </si>
+  <si>
+    <t>8075324258</t>
+  </si>
+  <si>
+    <t>New_Opp_ID</t>
+  </si>
+  <si>
+    <t>Customer_Name</t>
+  </si>
+  <si>
+    <t>CARPENTER INVESTMENTS (VINE STREET) LTD</t>
+  </si>
+  <si>
+    <t>CSV_File_1</t>
+  </si>
+  <si>
+    <t>Quote_ID</t>
+  </si>
+  <si>
+    <t>CSV_File_2</t>
+  </si>
+  <si>
+    <t>CSV_File_3</t>
+  </si>
+  <si>
+    <t>txs_File_1</t>
+  </si>
+  <si>
+    <t>COT_P1</t>
+  </si>
+  <si>
+    <t>txs_File_2</t>
+  </si>
+  <si>
+    <t>1171000000</t>
+  </si>
+  <si>
+    <t>txs_File_3</t>
+  </si>
+  <si>
+    <t>New_OPP_ID</t>
+  </si>
+  <si>
+    <t>txs_File_4</t>
+  </si>
+  <si>
+    <t>Premise</t>
+  </si>
+  <si>
+    <t>0246713154</t>
+  </si>
+  <si>
+    <t>Flex Basket</t>
+  </si>
+  <si>
+    <t>Person ID-1</t>
+  </si>
+  <si>
+    <t>Person ID-2</t>
+  </si>
+  <si>
+    <t>Person ID-3</t>
+  </si>
+  <si>
+    <t>Customer Upload file</t>
+  </si>
+  <si>
+    <t>Bulk Opp Uplaod</t>
+  </si>
+  <si>
+    <t>Opp ID-1</t>
+  </si>
+  <si>
+    <t>Opp ID-2</t>
+  </si>
+  <si>
+    <t>Opp ID-3</t>
+  </si>
+  <si>
+    <t>Quote ID-1</t>
+  </si>
+  <si>
+    <t>Quote ID-2</t>
+  </si>
+  <si>
+    <t>Quote ID-3</t>
+  </si>
+  <si>
+    <t>Structure Test Execution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earlier auomation executions were performed via a basic java setup due to TestNG access resrtictions, requiring manual local execution. With the setp of testNG and Maven-based framewrok, we now have structured test execution, better scalability, centralized dependency management, enhanced reporting, and readiness for parallel execution </t>
+  </si>
+  <si>
+    <t>Test Suite Management(.xml)</t>
+  </si>
+  <si>
+    <t>Reusability and scalability</t>
+  </si>
+  <si>
+    <t>Dedendency Management</t>
+  </si>
+  <si>
+    <t>Reporting &amp; Debugging</t>
+  </si>
+  <si>
+    <t>Parallel Execution Support</t>
+  </si>
+  <si>
+    <t>CI/CD</t>
+  </si>
+  <si>
+    <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S1_JAN_RT.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation2.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation3.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MediumFixed-p1\\Data_S7_RT.csv</t>
+  </si>
+  <si>
+    <t>Framework Id</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_1_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\AutomationDocuments\MCTOpportunity\OPP_2_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_3_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_4_feb_MCT 1 (2).txt</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CM-CUUB2_FLEX_BASKET_BV_30MAR2025 RT-BATCH 1.csv</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CMBLRNOP_S12_FLEX_ADDSITE_30March-2025 RT.csv</t>
+  </si>
+  <si>
+    <t>1560000000</t>
+  </si>
+  <si>
+    <t>6579077315</t>
+  </si>
+  <si>
+    <t>8525362589</t>
+  </si>
+  <si>
+    <t>Live Billing P1</t>
+  </si>
+  <si>
+    <t>Live Billing</t>
+  </si>
+  <si>
+    <t>Person_ID-1</t>
+  </si>
+  <si>
+    <t>Child Person ID</t>
+  </si>
+  <si>
+    <t>OPP_ID</t>
+  </si>
+  <si>
+    <t>NHH MPAN</t>
+  </si>
+  <si>
+    <t>HH MPAN</t>
+  </si>
+  <si>
+    <t>1502000000</t>
+  </si>
+  <si>
+    <t>5433000000</t>
+  </si>
+  <si>
     <t>4901343242  </t>
   </si>
   <si>
-    <t>UploadingFile</t>
-  </si>
-  <si>
-    <t>Premise_ID</t>
-  </si>
-  <si>
-    <t>7637797801</t>
-  </si>
-  <si>
-    <t>8075324258</t>
-  </si>
-  <si>
-    <t>New_Opp_ID</t>
-  </si>
-  <si>
-    <t>Customer_Name</t>
-  </si>
-  <si>
-    <t>CARPENTER INVESTMENTS (VINE STREET) LTD</t>
-  </si>
-  <si>
-    <t>CSV_File_1</t>
-  </si>
-  <si>
-    <t>Quote_ID</t>
-  </si>
-  <si>
-    <t>5876383266</t>
-  </si>
-  <si>
-    <t>4668211723</t>
-  </si>
-  <si>
-    <t>CSV_File_2</t>
-  </si>
-  <si>
-    <t>9337054612</t>
-  </si>
-  <si>
-    <t>CSV_File_3</t>
-  </si>
-  <si>
-    <t>txs_File_1</t>
-  </si>
-  <si>
-    <t>COT_P1</t>
-  </si>
-  <si>
-    <t>txs_File_2</t>
-  </si>
-  <si>
-    <t>1171000000</t>
-  </si>
-  <si>
-    <t>txs_File_3</t>
-  </si>
-  <si>
-    <t>New_OPP_ID</t>
-  </si>
-  <si>
-    <t>txs_File_4</t>
-  </si>
-  <si>
-    <t>Premise</t>
-  </si>
-  <si>
-    <t>0246713154</t>
-  </si>
-  <si>
-    <t>Flex Basket</t>
-  </si>
-  <si>
-    <t>Person ID-1</t>
-  </si>
-  <si>
-    <t>Person ID-2</t>
-  </si>
-  <si>
-    <t>Person ID-3</t>
-  </si>
-  <si>
-    <t>Customer Upload file</t>
-  </si>
-  <si>
-    <t>Bulk Opp Uplaod</t>
-  </si>
-  <si>
-    <t>Opp ID-1</t>
-  </si>
-  <si>
-    <t>Opp ID-2</t>
-  </si>
-  <si>
-    <t>Opp ID-3</t>
-  </si>
-  <si>
-    <t>Quote ID-1</t>
-  </si>
-  <si>
-    <t>Quote ID-2</t>
-  </si>
-  <si>
-    <t>Quote ID-3</t>
-  </si>
-  <si>
-    <t>Structure Test Execution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Earlier auomation executions were performed via a basic java setup due to TestNG access resrtictions, requiring manual local execution. With the setp of testNG and Maven-based framewrok, we now have structured test execution, better scalability, centralized dependency management, enhanced reporting, and readiness for parallel execution </t>
-  </si>
-  <si>
-    <t>Test Suite Management(.xml)</t>
-  </si>
-  <si>
-    <t>Reusability and scalability</t>
-  </si>
-  <si>
-    <t>Dedendency Management</t>
-  </si>
-  <si>
-    <t>Reporting &amp; Debugging</t>
-  </si>
-  <si>
-    <t>Parallel Execution Support</t>
-  </si>
-  <si>
-    <t>CI/CD</t>
-  </si>
-  <si>
-    <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S1_JAN_RT.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation2.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation3.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MediumFixed-p1\\Data_S7_RT.csv</t>
-  </si>
-  <si>
-    <t>Framework Id</t>
-  </si>
-  <si>
-    <t>0245182125</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_1_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\AutomationDocuments\MCTOpportunity\OPP_2_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_3_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\MCTOpportunity\\OPP_4_feb_MCT 1 (2).txt</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CM-CUUB2_FLEX_BASKET_BV_30MAR2025 RT-BATCH 1.csv</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\FlexBasket - P1\\Bhushan_CMBLRNOP_S12_FLEX_ADDSITE_30March-2025 RT.csv</t>
-  </si>
-  <si>
-    <t>1560000000</t>
-  </si>
-  <si>
-    <t>6579077315</t>
-  </si>
-  <si>
-    <t>8525362589</t>
-  </si>
-  <si>
-    <t>4565185268</t>
-  </si>
-  <si>
-    <t>6770510767</t>
-  </si>
-  <si>
-    <t>7730327480</t>
-  </si>
-  <si>
-    <t>8250985049</t>
-  </si>
-  <si>
-    <t>2633799055</t>
-  </si>
-  <si>
-    <t>5149622225</t>
-  </si>
-  <si>
-    <t>7777857402</t>
-  </si>
-  <si>
-    <t>Live Billing P1</t>
-  </si>
-  <si>
-    <t>Live Billing</t>
-  </si>
-  <si>
-    <t>Person_ID-1</t>
-  </si>
-  <si>
-    <t>Child Person ID</t>
-  </si>
-  <si>
-    <t>OPP_ID</t>
-  </si>
-  <si>
-    <t>NHH MPAN</t>
-  </si>
-  <si>
-    <t>HH MPAN</t>
-  </si>
-  <si>
-    <t>1502000000</t>
-  </si>
-  <si>
-    <t>5433000000</t>
-  </si>
-  <si>
-    <t>9574256063</t>
-  </si>
-  <si>
-    <t>6923383318</t>
-  </si>
-  <si>
-    <t>9759372210</t>
-  </si>
-  <si>
-    <t>0731479811</t>
-  </si>
-  <si>
-    <t>2696403742</t>
-  </si>
-  <si>
-    <t>2088160177</t>
-  </si>
-  <si>
-    <t>3149753310</t>
-  </si>
-  <si>
-    <t>2797082217</t>
-  </si>
-  <si>
-    <t>5591505466</t>
-  </si>
-  <si>
-    <t>4830622173</t>
-  </si>
-  <si>
-    <t>8252565730</t>
-  </si>
-  <si>
-    <t>8886735189</t>
-  </si>
-  <si>
-    <t>5077298692</t>
-  </si>
-  <si>
-    <t>6305334164</t>
-  </si>
-  <si>
-    <t>4327576054</t>
-  </si>
-  <si>
-    <t>2903614060</t>
-  </si>
-  <si>
-    <t>8654222347</t>
-  </si>
-  <si>
-    <t>2726673381</t>
-  </si>
-  <si>
-    <t>7033419122</t>
-  </si>
-  <si>
-    <t>1272705197</t>
-  </si>
-  <si>
-    <t>4011690183</t>
-  </si>
-  <si>
-    <t>1248446971</t>
-  </si>
-  <si>
-    <t>9869391872</t>
-  </si>
-  <si>
-    <t>5446917638</t>
-  </si>
-  <si>
-    <t>3027747152</t>
-  </si>
-  <si>
-    <t>6774312962</t>
-  </si>
-  <si>
-    <t>6716824684</t>
-  </si>
-  <si>
-    <t>3445934797</t>
-  </si>
-  <si>
-    <t>6748138279</t>
-  </si>
-  <si>
-    <t>1870397259</t>
-  </si>
-  <si>
-    <t>4804886734</t>
-  </si>
-  <si>
-    <t>3338983444</t>
-  </si>
-  <si>
-    <t>4471287196</t>
-  </si>
-  <si>
-    <t>6002003351</t>
-  </si>
-  <si>
-    <t>4907922041</t>
-  </si>
-  <si>
-    <t>4179721175</t>
-  </si>
-  <si>
-    <t>2541090599</t>
-  </si>
-  <si>
-    <t>7006261130</t>
-  </si>
-  <si>
-    <t>2388420562</t>
-  </si>
-  <si>
-    <t>9615984184</t>
-  </si>
-  <si>
-    <t>3365202343</t>
-  </si>
-  <si>
-    <t>3153018435</t>
-  </si>
-  <si>
-    <t>6993632357</t>
-  </si>
-  <si>
-    <t>7037655979</t>
-  </si>
-  <si>
-    <t>0076429936</t>
-  </si>
-  <si>
-    <t>3434630786</t>
-  </si>
-  <si>
-    <t>9804209447</t>
-  </si>
-  <si>
-    <t>4777532563</t>
-  </si>
-  <si>
-    <t>6794678807</t>
-  </si>
-  <si>
-    <t>3150483671</t>
-  </si>
-  <si>
-    <t>5375000455</t>
-  </si>
-  <si>
-    <t>7935933322</t>
-  </si>
-  <si>
-    <t>8832122010</t>
-  </si>
-  <si>
-    <t>8818211609</t>
-  </si>
-  <si>
-    <t>0171186953</t>
-  </si>
-  <si>
-    <t>6841200765</t>
+    <t>0088592004</t>
+  </si>
+  <si>
+    <t>9416177446</t>
+  </si>
+  <si>
+    <t>2064721790</t>
+  </si>
+  <si>
+    <t>8593051363</t>
+  </si>
+  <si>
+    <t>8967788332</t>
+  </si>
+  <si>
+    <t>1237124980</t>
+  </si>
+  <si>
+    <t>2657637606</t>
+  </si>
+  <si>
+    <t>8330422730</t>
+  </si>
+  <si>
+    <t>4377885532</t>
+  </si>
+  <si>
+    <t>7223786676</t>
+  </si>
+  <si>
+    <t>3668941872</t>
+  </si>
+  <si>
+    <t>1376326608</t>
+  </si>
+  <si>
+    <t>1895143104</t>
+  </si>
+  <si>
+    <t>3288881535</t>
+  </si>
+  <si>
+    <t>9505162772</t>
+  </si>
+  <si>
+    <t>1294486442</t>
+  </si>
+  <si>
+    <t>6501846304</t>
+  </si>
+  <si>
+    <t>2317209141</t>
+  </si>
+  <si>
+    <t>0168625971</t>
+  </si>
+  <si>
+    <t>2020328319</t>
   </si>
 </sst>
 </file>
@@ -574,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -593,6 +452,9 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -602,8 +464,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1099,23 +961,23 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12"/>
+      <c r="G1" s="13"/>
       <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="12"/>
+      <c r="J1" s="13"/>
       <c r="O1" s="9" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1131,8 +993,8 @@
       <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="15" t="s">
-        <v>67</v>
+      <c r="E2" s="12" t="s">
+        <v>62</v>
       </c>
       <c r="F2" s="2">
         <v>3151000000</v>
@@ -1141,171 +1003,171 @@
         <v>4903000000</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>11</v>
-      </c>
       <c r="J2" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="F3" s="2">
-        <v>2280000000</v>
+        <v>7481000527</v>
       </c>
       <c r="G3" s="2">
         <v>3482055476</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="I3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="J5" s="16">
+        <v>7013475671</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D6" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H6" s="2">
-        <v>7007727568</v>
+        <v>9402999903</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D7" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D8" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D9" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D10" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H11" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G12" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H12" s="2">
         <v>7641311796</v>
@@ -1314,10 +1176,10 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
       <c r="E13" s="10" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H13" s="2">
         <v>9065870431</v>
@@ -1325,13 +1187,13 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D14" s="1" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="H14" s="2">
         <v>4376617890</v>
@@ -1339,90 +1201,90 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D15" s="1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D16" s="1" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>141</v>
+        <v>78</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D17" s="1" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E17" s="11">
         <v>1591062611809</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E18" s="11">
         <v>1600000042214</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G19" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G20" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G21" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G22" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G23" s="8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -1447,11 +1309,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1473,47 +1335,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>47</v>
+        <v>42</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="14"/>
+        <v>44</v>
+      </c>
+      <c r="B2" s="15"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="14"/>
+        <v>45</v>
+      </c>
+      <c r="B3" s="15"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="14"/>
+        <v>46</v>
+      </c>
+      <c r="B4" s="15"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="14"/>
+        <v>47</v>
+      </c>
+      <c r="B5" s="15"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="14"/>
+        <v>48</v>
+      </c>
+      <c r="B6" s="15"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="14"/>
+        <v>49</v>
+      </c>
+      <c r="B7" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
updated with comc15 p2 & COMC16P2
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1890684E-1950-4984-9E00-5D3817C51ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF1D931-92A6-45AB-8B67-72A89BD2C40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -229,12 +229,6 @@
     <t>1560000000</t>
   </si>
   <si>
-    <t>6579077315</t>
-  </si>
-  <si>
-    <t>8525362589</t>
-  </si>
-  <si>
     <t>Live Billing P1</t>
   </si>
   <si>
@@ -265,24 +259,9 @@
     <t>4901343242  </t>
   </si>
   <si>
-    <t>0088592004</t>
-  </si>
-  <si>
-    <t>9416177446</t>
-  </si>
-  <si>
-    <t>2064721790</t>
-  </si>
-  <si>
     <t>8593051363</t>
   </si>
   <si>
-    <t>8967788332</t>
-  </si>
-  <si>
-    <t>1237124980</t>
-  </si>
-  <si>
     <t>2657637606</t>
   </si>
   <si>
@@ -295,34 +274,43 @@
     <t>7223786676</t>
   </si>
   <si>
-    <t>3668941872</t>
-  </si>
-  <si>
-    <t>1376326608</t>
-  </si>
-  <si>
-    <t>1895143104</t>
-  </si>
-  <si>
-    <t>3288881535</t>
-  </si>
-  <si>
-    <t>9505162772</t>
-  </si>
-  <si>
-    <t>1294486442</t>
-  </si>
-  <si>
-    <t>6501846304</t>
-  </si>
-  <si>
-    <t>2317209141</t>
-  </si>
-  <si>
-    <t>0168625971</t>
-  </si>
-  <si>
-    <t>2020328319</t>
+    <t>5788655316</t>
+  </si>
+  <si>
+    <t>7383143448</t>
+  </si>
+  <si>
+    <t>4104294675</t>
+  </si>
+  <si>
+    <t>0454438612</t>
+  </si>
+  <si>
+    <t>0868221199</t>
+  </si>
+  <si>
+    <t>4889000061</t>
+  </si>
+  <si>
+    <t>3151000000</t>
+  </si>
+  <si>
+    <t>1091205047</t>
+  </si>
+  <si>
+    <t>4903000000</t>
+  </si>
+  <si>
+    <t>5183752121</t>
+  </si>
+  <si>
+    <t>8298601988</t>
+  </si>
+  <si>
+    <t>8052186083</t>
+  </si>
+  <si>
+    <t>3027972116</t>
   </si>
 </sst>
 </file>
@@ -330,7 +318,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -397,6 +385,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF312D2A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -433,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -455,6 +449,9 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -464,7 +461,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -961,23 +961,23 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13" t="s">
+      <c r="E1" s="14"/>
+      <c r="F1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="13"/>
+      <c r="G1" s="14"/>
       <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="13"/>
+      <c r="J1" s="14"/>
       <c r="O1" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -996,14 +996,14 @@
       <c r="E2" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="2">
-        <v>3151000000</v>
-      </c>
-      <c r="G2" s="2">
-        <v>4903000000</v>
+      <c r="F2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>10</v>
@@ -1026,7 +1026,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="F3" s="2">
         <v>7481000527</v>
@@ -1048,31 +1048,37 @@
       <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" s="2"/>
+      <c r="B4" s="2">
+        <v>7603082575</v>
+      </c>
+      <c r="C4" s="17">
+        <v>5627576502</v>
+      </c>
       <c r="D4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="H4" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>75</v>
+      <c r="B5" s="18">
+        <v>9385974501</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>19</v>
@@ -1081,12 +1087,12 @@
         <v>52</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="16">
+      <c r="J5" s="13">
         <v>7013475671</v>
       </c>
     </row>
@@ -1098,7 +1104,7 @@
         <v>53</v>
       </c>
       <c r="H6" s="2">
-        <v>9402999903</v>
+        <v>6387246001</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1137,7 +1143,7 @@
         <v>26</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1162,7 +1168,7 @@
         <v>18</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -1176,7 +1182,7 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
       <c r="E13" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>32</v>
@@ -1187,10 +1193,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D14" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>33</v>
@@ -1201,10 +1207,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D15" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>34</v>
@@ -1215,10 +1221,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D16" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>35</v>
@@ -1229,7 +1235,7 @@
     </row>
     <row r="17" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D17" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E17" s="11">
         <v>1591062611809</v>
@@ -1238,12 +1244,12 @@
         <v>36</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E18" s="11">
         <v>1600000042214</v>
@@ -1252,7 +1258,7 @@
         <v>37</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="4:8" x14ac:dyDescent="0.25">
@@ -1260,7 +1266,7 @@
         <v>38</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.25">
@@ -1268,7 +1274,7 @@
         <v>55</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="4:8" x14ac:dyDescent="0.25">
@@ -1309,11 +1315,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1337,7 +1343,7 @@
       <c r="A1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1345,37 +1351,37 @@
       <c r="A2" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="16"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="15"/>
+      <c r="B3" s="16"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="15"/>
+      <c r="B4" s="16"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="15"/>
+      <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="15"/>
+      <c r="B6" s="16"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="15"/>
+      <c r="B7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
commit with new connection update
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="118">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -311,6 +311,87 @@
   </si>
   <si>
     <t>3027972116</t>
+  </si>
+  <si>
+    <t>1226625461</t>
+  </si>
+  <si>
+    <t>9370786868</t>
+  </si>
+  <si>
+    <t>4027493752</t>
+  </si>
+  <si>
+    <t>2374281638</t>
+  </si>
+  <si>
+    <t>3462929859</t>
+  </si>
+  <si>
+    <t>1325562981</t>
+  </si>
+  <si>
+    <t>0448141470</t>
+  </si>
+  <si>
+    <t>8883877545</t>
+  </si>
+  <si>
+    <t>9425380155</t>
+  </si>
+  <si>
+    <t>8310412047</t>
+  </si>
+  <si>
+    <t>9958182088</t>
+  </si>
+  <si>
+    <t>1771063571</t>
+  </si>
+  <si>
+    <t>4650206388</t>
+  </si>
+  <si>
+    <t>8365807128</t>
+  </si>
+  <si>
+    <t>1055876824</t>
+  </si>
+  <si>
+    <t>5993391500</t>
+  </si>
+  <si>
+    <t>2852035984</t>
+  </si>
+  <si>
+    <t>0680917203</t>
+  </si>
+  <si>
+    <t>3596749555</t>
+  </si>
+  <si>
+    <t>8402952021</t>
+  </si>
+  <si>
+    <t>9987780391</t>
+  </si>
+  <si>
+    <t>0484722268</t>
+  </si>
+  <si>
+    <t>7458080547</t>
+  </si>
+  <si>
+    <t>6938939265</t>
+  </si>
+  <si>
+    <t>5436745595</t>
+  </si>
+  <si>
+    <t>3814067775</t>
+  </si>
+  <si>
+    <t>1197705291</t>
   </si>
 </sst>
 </file>
@@ -1061,13 +1142,13 @@
         <v>51</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1087,7 +1168,7 @@
         <v>52</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>18</v>
@@ -1143,7 +1224,7 @@
         <v>26</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1168,7 +1249,7 @@
         <v>18</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated with NewConnection error
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="154">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -392,6 +392,114 @@
   </si>
   <si>
     <t>1197705291</t>
+  </si>
+  <si>
+    <t>6067902145</t>
+  </si>
+  <si>
+    <t>1397144388</t>
+  </si>
+  <si>
+    <t>0522738808</t>
+  </si>
+  <si>
+    <t>4078657946</t>
+  </si>
+  <si>
+    <t>7994206658</t>
+  </si>
+  <si>
+    <t>3053062524</t>
+  </si>
+  <si>
+    <t>5957934712</t>
+  </si>
+  <si>
+    <t>2719749931</t>
+  </si>
+  <si>
+    <t>4639673826</t>
+  </si>
+  <si>
+    <t>8957206800</t>
+  </si>
+  <si>
+    <t>1349058026</t>
+  </si>
+  <si>
+    <t>9019098670</t>
+  </si>
+  <si>
+    <t>1087548124</t>
+  </si>
+  <si>
+    <t>8116405369</t>
+  </si>
+  <si>
+    <t>4824312402</t>
+  </si>
+  <si>
+    <t>1837895607</t>
+  </si>
+  <si>
+    <t>8104180362</t>
+  </si>
+  <si>
+    <t>3158503702</t>
+  </si>
+  <si>
+    <t>7042957423</t>
+  </si>
+  <si>
+    <t>3767468561</t>
+  </si>
+  <si>
+    <t>0001277004</t>
+  </si>
+  <si>
+    <t>3962389420</t>
+  </si>
+  <si>
+    <t>3910227242</t>
+  </si>
+  <si>
+    <t>3421442758</t>
+  </si>
+  <si>
+    <t>0135892978</t>
+  </si>
+  <si>
+    <t>6704969355</t>
+  </si>
+  <si>
+    <t>8601835224</t>
+  </si>
+  <si>
+    <t>2162560901</t>
+  </si>
+  <si>
+    <t>1731376266</t>
+  </si>
+  <si>
+    <t>0293386730</t>
+  </si>
+  <si>
+    <t>2610211262</t>
+  </si>
+  <si>
+    <t>7475707708</t>
+  </si>
+  <si>
+    <t>3840025956</t>
+  </si>
+  <si>
+    <t>8054053342</t>
+  </si>
+  <si>
+    <t>3170077325</t>
+  </si>
+  <si>
+    <t>0864235659</t>
   </si>
 </sst>
 </file>
@@ -1142,10 +1250,10 @@
         <v>51</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>117</v>
+        <v>153</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>98</v>
@@ -1224,7 +1332,7 @@
         <v>26</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1249,7 +1357,7 @@
         <v>18</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
commiting before email automation
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD31D4C3-6094-4E83-9111-2970253A0430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{210F53E8-A16F-47C3-A247-188481F8E07E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="99">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -76,9 +76,6 @@
     <t>Premise_ID</t>
   </si>
   <si>
-    <t>7637797801</t>
-  </si>
-  <si>
     <t>8075324258</t>
   </si>
   <si>
@@ -259,24 +256,9 @@
     <t>4901343242  </t>
   </si>
   <si>
-    <t>2657637606</t>
-  </si>
-  <si>
-    <t>8330422730</t>
-  </si>
-  <si>
-    <t>4377885532</t>
-  </si>
-  <si>
-    <t>7223786676</t>
-  </si>
-  <si>
     <t>4104294675</t>
   </si>
   <si>
-    <t>4889000061</t>
-  </si>
-  <si>
     <t>3151000000</t>
   </si>
   <si>
@@ -286,12 +268,6 @@
     <t>1647142826</t>
   </si>
   <si>
-    <t>9107254520</t>
-  </si>
-  <si>
-    <t>7064260282</t>
-  </si>
-  <si>
     <t>7477463648</t>
   </si>
   <si>
@@ -307,64 +283,58 @@
     <t>Opportunity ID</t>
   </si>
   <si>
-    <t>5221215146</t>
-  </si>
-  <si>
-    <t>0748189416</t>
-  </si>
-  <si>
-    <t>7294457977</t>
-  </si>
-  <si>
-    <t>2084961921</t>
-  </si>
-  <si>
-    <t>9328330186</t>
-  </si>
-  <si>
-    <t>3237380237</t>
-  </si>
-  <si>
-    <t>4302254944</t>
-  </si>
-  <si>
-    <t>2203927699</t>
-  </si>
-  <si>
-    <t>5457668088</t>
-  </si>
-  <si>
-    <t>9724826246</t>
-  </si>
-  <si>
-    <t>9465071728</t>
-  </si>
-  <si>
-    <t>8884241383</t>
-  </si>
-  <si>
-    <t>1608228787</t>
-  </si>
-  <si>
-    <t>2295122924</t>
-  </si>
-  <si>
-    <t>4149562822</t>
-  </si>
-  <si>
-    <t>5129166392</t>
-  </si>
-  <si>
-    <t>3205132883</t>
-  </si>
-  <si>
-    <t>9104217704</t>
-  </si>
-  <si>
-    <t>2475479013</t>
-  </si>
-  <si>
-    <t>6403155009</t>
+    <t>9502355347</t>
+  </si>
+  <si>
+    <t>7854917024</t>
+  </si>
+  <si>
+    <t>3603800045</t>
+  </si>
+  <si>
+    <t>5334047124</t>
+  </si>
+  <si>
+    <t>8150883921</t>
+  </si>
+  <si>
+    <t>0237734270</t>
+  </si>
+  <si>
+    <t>6792331839</t>
+  </si>
+  <si>
+    <t>1659100631</t>
+  </si>
+  <si>
+    <t>3799751984</t>
+  </si>
+  <si>
+    <t>0767706356</t>
+  </si>
+  <si>
+    <t>2614736311</t>
+  </si>
+  <si>
+    <t>4018224261</t>
+  </si>
+  <si>
+    <t>7253642895</t>
+  </si>
+  <si>
+    <t>3229770534</t>
+  </si>
+  <si>
+    <t>4119925628</t>
+  </si>
+  <si>
+    <t>4684174886</t>
+  </si>
+  <si>
+    <t>1722634350</t>
+  </si>
+  <si>
+    <t>9775788338</t>
   </si>
 </sst>
 </file>
@@ -512,6 +482,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -521,7 +492,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1016,23 +986,23 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16" t="s">
+      <c r="E1" s="17"/>
+      <c r="F1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="16"/>
+      <c r="G1" s="17"/>
       <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="16"/>
+      <c r="J1" s="17"/>
       <c r="O1" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1049,39 +1019,39 @@
         <v>7</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="2">
+        <v>2542811529</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="F3" s="2">
         <v>7481000527</v>
@@ -1090,79 +1060,79 @@
         <v>3482055476</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="2">
-        <v>7603082575</v>
-      </c>
-      <c r="C4" s="14">
-        <v>5627576502</v>
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>91</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="J4" s="19" t="s">
-        <v>108</v>
+        <v>80</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="6">
+        <v>5003067576</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="15">
-        <v>9385974501</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>19</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="13" t="s">
         <v>85</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D6" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H6" s="2">
         <v>8883877545</v>
@@ -1170,71 +1140,71 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D8" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="J9" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="I10" s="5" t="s">
+      <c r="J10" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H11" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G12" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H12" s="2">
         <v>7641311796</v>
@@ -1243,10 +1213,10 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
       <c r="E13" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H13" s="2">
         <v>9065870431</v>
@@ -1254,13 +1224,13 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D14" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H14" s="2">
         <v>4376617890</v>
@@ -1268,90 +1238,90 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D15" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D16" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D17" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E17" s="11">
         <v>1591062611809</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E18" s="11">
         <v>1600000042214</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G19" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G20" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G21" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G22" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G23" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -1376,11 +1346,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1402,47 +1372,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>42</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="18"/>
+        <v>43</v>
+      </c>
+      <c r="B2" s="19"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="18"/>
+        <v>44</v>
+      </c>
+      <c r="B3" s="19"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="18"/>
+        <v>45</v>
+      </c>
+      <c r="B4" s="19"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="18"/>
+        <v>46</v>
+      </c>
+      <c r="B5" s="19"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="18"/>
+        <v>47</v>
+      </c>
+      <c r="B6" s="19"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="18"/>
+        <v>48</v>
+      </c>
+      <c r="B7" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
commit with random name
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64B0CDCC-E8B8-4257-A2E7-2CB29245A80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246D2D3F-5683-4873-BE37-62EFCF08C25F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -82,9 +82,6 @@
     <t>Customer_Name</t>
   </si>
   <si>
-    <t>CARPENTER INVESTMENTS (VINE STREET) LTD</t>
-  </si>
-  <si>
     <t>CSV_File_1</t>
   </si>
   <si>
@@ -184,9 +181,6 @@
     <t>CI/CD</t>
   </si>
   <si>
-    <t>C:\\Users\\srina1k\\OneDrive - EDF\\Data_S1_JAN_RT.csv</t>
-  </si>
-  <si>
     <t>C:\\AutomationDocuments\\MCTOpportunity\\OpportunityCreation1.csv</t>
   </si>
   <si>
@@ -289,83 +283,40 @@
     <t>5334047124</t>
   </si>
   <si>
-    <t>8150883921</t>
-  </si>
-  <si>
-    <t>0237734270</t>
-  </si>
-  <si>
-    <t>3799751984</t>
-  </si>
-  <si>
-    <t>0767706356</t>
-  </si>
-  <si>
     <t>2614736311</t>
   </si>
   <si>
     <t>3229770534</t>
   </si>
   <si>
-    <t>5919937840</t>
-  </si>
-  <si>
-    <t>9253201165</t>
-  </si>
-  <si>
     <t>0251000000</t>
   </si>
   <si>
-    <t>6533175242</t>
-  </si>
-  <si>
     <t>2768212218</t>
   </si>
   <si>
     <t>1687810020</t>
   </si>
   <si>
-    <t>8561982918</t>
-  </si>
-  <si>
-    <t>8640658772</t>
-  </si>
-  <si>
-    <t>2451718056</t>
-  </si>
-  <si>
-    <t>1186422616</t>
-  </si>
-  <si>
-    <t>2621111120</t>
-  </si>
-  <si>
-    <t>2885046657</t>
-  </si>
-  <si>
-    <t>1846541188</t>
-  </si>
-  <si>
-    <t>6676146057</t>
-  </si>
-  <si>
-    <t>8257553204</t>
-  </si>
-  <si>
-    <t>4956031316</t>
-  </si>
-  <si>
-    <t>5503095233</t>
-  </si>
-  <si>
-    <t>4845824404</t>
+    <t>APEX HOTELS LIMITED</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\smallFixed-p1\\smallFixed_anotherfile.txt</t>
+  </si>
+  <si>
+    <t>4366972111</t>
+  </si>
+  <si>
+    <t>7129104328</t>
+  </si>
+  <si>
+    <t>2538445686</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -985,19 +936,19 @@
   <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="2" max="2" customWidth="true" width="15.0"/>
-    <col min="3" max="3" customWidth="true" width="12.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="14.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="52.140625"/>
-    <col min="6" max="6" customWidth="true" width="17.140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="20.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="51.28515625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="47.5703125"/>
-    <col min="12" max="12" customWidth="true" width="5.85546875"/>
-    <col min="13" max="14" customWidth="true" hidden="true" width="9.140625"/>
-    <col min="15" max="15" customWidth="true" width="24.85546875"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="51.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.85546875" customWidth="1"/>
+    <col min="13" max="14" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1026,7 +977,7 @@
       </c>
       <c r="J1" s="17"/>
       <c r="O1" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1034,7 +985,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>8</v>
@@ -1043,22 +994,22 @@
         <v>7</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1075,7 +1026,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="F3" s="2">
         <v>7481000527</v>
@@ -1083,14 +1034,14 @@
       <c r="G3" s="2">
         <v>3482055476</v>
       </c>
-      <c r="H3" t="s" s="0">
-        <v>52</v>
+      <c r="H3" t="s">
+        <v>50</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1098,65 +1049,65 @@
         <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="C5" s="6">
         <v>5003067576</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>104</v>
+        <v>15</v>
+      </c>
+      <c r="J5" s="13">
+        <v>2163704004</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D6" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H6" s="2">
         <v>8883877545</v>
@@ -1164,71 +1115,71 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D8" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="J9" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="I10" s="5" t="s">
+      <c r="J10" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H11" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G12" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H12" s="2">
         <v>7641311796</v>
@@ -1237,10 +1188,10 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
       <c r="E13" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H13" s="2">
         <v>9065870431</v>
@@ -1248,13 +1199,13 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D14" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H14" s="2">
         <v>4376617890</v>
@@ -1262,90 +1213,90 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D15" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D16" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D17" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E17" s="11">
         <v>1591062611809</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E18" s="11">
         <v>1600000042214</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G19" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G20" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G21" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G22" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="4:8" x14ac:dyDescent="0.25">
       <c r="G23" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -1366,7 +1317,7 @@
   <dimension ref="C1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="9.140625"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
@@ -1390,51 +1341,51 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="28.140625"/>
-    <col min="2" max="2" customWidth="true" width="56.28515625"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="56.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>40</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" s="19"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="19"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="19"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" s="19"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="19"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" s="19"/>
     </row>

</xml_diff>

<commit_message>
updated with entity creation
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="103">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -311,12 +311,49 @@
   </si>
   <si>
     <t>2538445686</t>
+  </si>
+  <si>
+    <t>9857259485</t>
+  </si>
+  <si>
+    <t>7197589391</t>
+  </si>
+  <si>
+    <t>9681609259</t>
+  </si>
+  <si>
+    <t>5245411146</t>
+  </si>
+  <si>
+    <t>4028304572</t>
+  </si>
+  <si>
+    <t>5734176517</t>
+  </si>
+  <si>
+    <t>1735464039</t>
+  </si>
+  <si>
+    <t>6629923603</t>
+  </si>
+  <si>
+    <t>1679359718</t>
+  </si>
+  <si>
+    <t>9643483140</t>
+  </si>
+  <si>
+    <t>7241743548</t>
+  </si>
+  <si>
+    <t>6204668662</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -936,19 +973,19 @@
   <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.140625" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="47.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" customWidth="1"/>
-    <col min="13" max="14" width="9.140625" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="24.85546875" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="2" max="2" customWidth="true" width="15.0"/>
+    <col min="3" max="3" customWidth="true" width="12.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="14.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="52.140625"/>
+    <col min="6" max="6" customWidth="true" width="17.140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="20.140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="51.28515625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="47.5703125"/>
+    <col min="12" max="12" customWidth="true" width="5.85546875"/>
+    <col min="13" max="14" customWidth="true" hidden="true" width="9.140625"/>
+    <col min="15" max="15" customWidth="true" width="24.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1034,7 +1071,7 @@
       <c r="G3" s="2">
         <v>3482055476</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" t="s" s="0">
         <v>50</v>
       </c>
       <c r="I3" s="5" t="s">
@@ -1061,10 +1098,10 @@
         <v>47</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>72</v>
@@ -1317,7 +1354,7 @@
   <dimension ref="C1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
@@ -1341,8 +1378,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.140625" customWidth="1"/>
-    <col min="2" max="2" width="56.28515625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="28.140625"/>
+    <col min="2" max="2" customWidth="true" width="56.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated with comc15 errors
</commit_message>
<xml_diff>
--- a/src/main/java/Resources/RTScenarioTestDataReport.xlsx
+++ b/src/main/java/Resources/RTScenarioTestDataReport.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srina1k\IdeaProjects\C2MUpGradeAutomation\src\main\java\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F08D8E-2B37-4DF2-9F96-DF271E368817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D796B5D0-20C8-4D2E-B432-ED7CBB9C885C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="90">
   <si>
     <t>Sceanrio_name</t>
   </si>
@@ -277,9 +277,6 @@
     <t>5334047124</t>
   </si>
   <si>
-    <t>2614736311</t>
-  </si>
-  <si>
     <t>3229770534</t>
   </si>
   <si>
@@ -289,80 +286,34 @@
     <t>1687810020</t>
   </si>
   <si>
-    <t>APEX HOTELS LIMITED</t>
-  </si>
-  <si>
-    <t>C:\\AutomationDocuments\\smallFixed-p1\\smallFixed_anotherfile.txt</t>
-  </si>
-  <si>
-    <t>4366972111</t>
-  </si>
-  <si>
-    <t>1280017495</t>
-  </si>
-  <si>
-    <t>3120741011</t>
-  </si>
-  <si>
     <t>5024444444</t>
   </si>
   <si>
-    <t>8696737494</t>
-  </si>
-  <si>
-    <t>4723679856</t>
-  </si>
-  <si>
-    <t>8107777073</t>
-  </si>
-  <si>
-    <t>0540283571</t>
-  </si>
-  <si>
-    <t>9698138967</t>
-  </si>
-  <si>
-    <t>6224821295</t>
-  </si>
-  <si>
-    <t>8174780567</t>
-  </si>
-  <si>
     <t>7046751109</t>
   </si>
   <si>
     <t>1115548988</t>
   </si>
   <si>
-    <t>8425034442</t>
-  </si>
-  <si>
-    <t>0796704936</t>
-  </si>
-  <si>
-    <t>4746281339</t>
-  </si>
-  <si>
-    <t>2238870816</t>
-  </si>
-  <si>
-    <t>0682337472</t>
-  </si>
-  <si>
-    <t>2955907747</t>
-  </si>
-  <si>
-    <t>3764822237</t>
-  </si>
-  <si>
-    <t>7929650343</t>
+    <t>1316752250</t>
+  </si>
+  <si>
+    <t>0420829170</t>
+  </si>
+  <si>
+    <t>C:\\AutomationDocuments\\smallFixed-p1\\smallfixed1.txt</t>
+  </si>
+  <si>
+    <t>Sussex Partnership Nhs Foundation Trust</t>
+  </si>
+  <si>
+    <t>9283789408</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -982,19 +933,19 @@
   <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="2" max="2" customWidth="true" width="15.0"/>
-    <col min="3" max="3" customWidth="true" width="12.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="14.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="52.140625"/>
-    <col min="6" max="6" customWidth="true" width="17.140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="20.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="51.28515625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="47.5703125"/>
-    <col min="12" max="12" customWidth="true" width="5.85546875"/>
-    <col min="13" max="14" customWidth="true" hidden="true" width="9.140625"/>
-    <col min="15" max="15" customWidth="true" width="24.85546875"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="51.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.85546875" customWidth="1"/>
+    <col min="13" max="14" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1031,10 +982,10 @@
         <v>7</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>7</v>
@@ -1055,7 +1006,7 @@
         <v>8</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1072,7 +1023,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F3" s="2">
         <v>7481000527</v>
@@ -1080,14 +1031,14 @@
       <c r="G3" s="2">
         <v>3482055476</v>
       </c>
-      <c r="H3" t="s" s="0">
+      <c r="H3" t="s">
         <v>48</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1098,7 +1049,7 @@
         <v>2768212218</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>12</v>
@@ -1107,10 +1058,10 @@
         <v>45</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>70</v>
@@ -1119,7 +1070,7 @@
         <v>74</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1127,10 +1078,10 @@
         <v>13</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>14</v>
@@ -1145,7 +1096,7 @@
         <v>13</v>
       </c>
       <c r="J5" s="13">
-        <v>2163704004</v>
+        <v>6804661350</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1363,7 +1314,7 @@
   <dimension ref="C1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="9.140625"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
@@ -1387,8 +1338,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="28.140625"/>
-    <col min="2" max="2" customWidth="true" width="56.28515625"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="56.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>